<commit_message>
Auto update (2026-05-06 11:28:37) | Files: app.js node_down.xlsx ~$node_down.xlsx
</commit_message>
<xml_diff>
--- a/node_down.xlsx
+++ b/node_down.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:J86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -538,7 +538,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>18:41:48</t>
+          <t>19:40:19</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
@@ -590,7 +590,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>17:12:26</t>
+          <t>18:10:57</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -612,12 +612,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AC943</t>
+          <t>IM036</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CARR_SEGUELA</t>
+          <t>SEGUELA_RTE_BOLO</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -627,22 +627,22 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>AC943</t>
+          <t>SEGUELA_ROUTE_BOLO</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>BTS OUTAGE HUA</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-05-05 20:01:07</t>
+          <t>2026-05-05 20:04:10</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>14:05:24</t>
+          <t>15:00:52</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
@@ -664,12 +664,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>IM036</t>
+          <t>AC943</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SEGUELA_RTE_BOLO</t>
+          <t>CARR_SEGUELA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -679,7 +679,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>SEGUELA_ROUTE_BOLO</t>
+          <t>CARR_SEGUELA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -689,12 +689,12 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-05-05 20:04:10</t>
+          <t>2026-05-05 20:04:33</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>14:02:21</t>
+          <t>15:00:29</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -716,12 +716,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>AC943</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CARR_SEGUELA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CARR_SEGUELA</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -741,12 +741,12 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-05-05 20:04:33</t>
+          <t>2026-05-05 22:36:33</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>14:01:58</t>
+          <t>12:28:29</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
@@ -756,24 +756,24 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>NO DG</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>ET803</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>ABOBO_AVOCATIER_2 CHATEAUX</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -783,49 +783,49 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>BB_ET803_GL</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>Heartbeat Failure</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-05-05 22:36:33</t>
+          <t>2026-05-06 04:19:07</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>11:29:58</t>
+          <t>06:45:55</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>NO DG</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ET803</t>
+          <t>ET584</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ABOBO_AVOCATIER_2 CHATEAUX</t>
+          <t>PRUNELLE_JACQUEVIL</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>BB_ET803_GL</t>
+          <t>BB_ET584_GL</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -845,12 +845,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-05-06 04:19:07</t>
+          <t>2026-05-06 07:10:24</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>05:47:24</t>
+          <t>04:40:21</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -867,17 +867,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>AC178</t>
+          <t>ET416</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>AGNIKRO</t>
+          <t>SAGBE_CELESTE</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>BB_AC178_GL</t>
+          <t>BB_ET416_GL</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -897,12 +897,12 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-05-06 05:19:21</t>
+          <t>2026-05-06 07:18:08</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>04:47:10</t>
+          <t>03:46:54</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -912,24 +912,24 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>NO DG</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>ET504</t>
+          <t>AC334</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>ZEPREGUHE</t>
+          <t>STIF</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -939,49 +939,49 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>ZEBREZIHE</t>
+          <t>BB_AC334_GL</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>Heartbeat Failure</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-05-06 06:38:09</t>
+          <t>2026-05-06 08:00:27</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>03:28:22</t>
+          <t>03:04:35</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>NO DG</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>AC137</t>
+          <t>ET402</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>DAL_ESCADRON</t>
+          <t>ADJAME_UTB</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -991,27 +991,27 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>DAL_ESCADRON</t>
+          <t>BB_ET402_GL</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>Heartbeat Failure</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>2026-05-06 06:56:41</t>
+          <t>2026-05-06 08:02:43</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>03:09:50</t>
+          <t>03:02:19</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1028,12 +1028,12 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ET584</t>
+          <t>ET293</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>PRUNELLE_JACQUEVIL</t>
+          <t>NDJEM</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>BB_ET584_GL</t>
+          <t>BB_ET293_GL</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>ENODEB OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>2026-05-06 07:10:24</t>
+          <t>2026-05-06 08:37:47</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>03:41:50</t>
+          <t>02:29:40</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1075,17 +1075,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ET416</t>
+          <t>AC333</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>SAGBE_CELESTE</t>
+          <t>DJEDA</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1095,7 +1095,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>BB_ET416_GL</t>
+          <t>BB_AC333_GL</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -1105,12 +1105,12 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>2026-05-06 07:18:08</t>
+          <t>2026-05-06 09:09:45</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>02:48:23</t>
+          <t>01:55:17</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
@@ -1127,17 +1127,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ET816</t>
+          <t>AC965</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>MASSADOUGOU_EST</t>
+          <t>DIOGOBOUA</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1147,22 +1147,22 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>BB_ET816_GL</t>
+          <t>AC965_900</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>BTS OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>2026-05-06 07:29:58</t>
+          <t>2026-05-06 09:26:09</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>02:36:33</t>
+          <t>01:38:53</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1172,24 +1172,24 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>NO DG</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>AC334</t>
+          <t>ET567</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>STIF</t>
+          <t>BKE_CAMPUS2</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -1199,32 +1199,32 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>BB_AC334_GL</t>
+          <t>BKE_CAMPUS2</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>2026-05-06 08:00:27</t>
+          <t>2026-05-06 09:30:23</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>02:06:04</t>
+          <t>01:34:39</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>NO DG</t>
         </is>
       </c>
     </row>
@@ -1236,12 +1236,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ET402</t>
+          <t>ET019</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>ADJAME_UTB</t>
+          <t>BLACK_MARKET</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1251,7 +1251,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>BB_ET402_GL</t>
+          <t>BB_ET019_GL</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1261,12 +1261,12 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>2026-05-06 08:02:43</t>
+          <t>2026-05-06 09:54:55</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>02:03:48</t>
+          <t>01:10:07</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -1283,17 +1283,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ET293</t>
+          <t>ET641</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>NDJEM</t>
+          <t>DIANGOBO</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -1303,22 +1303,22 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>BB_ET293_GL</t>
+          <t>BB_ET641_GL</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>ENODEB OUTAGE ERIC</t>
+          <t>Heartbeat Failure</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2026-05-06 08:37:47</t>
+          <t>2026-05-06 10:04:22</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>01:31:09</t>
+          <t>01:00:40</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1335,17 +1335,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ET350</t>
+          <t>IM289</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BOUAFLE_HERE</t>
+          <t>KOLIKO</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1355,7 +1355,7 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>BOUAFLE_HERE</t>
+          <t>KOLIKO</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1365,12 +1365,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>2026-05-06 08:49:23</t>
+          <t>2026-05-06 10:04:50</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>01:17:08</t>
+          <t>01:00:12</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1387,17 +1387,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>AC333</t>
+          <t>IM398</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DJEDA</t>
+          <t>RURAL_ALLUIMINANKRO</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1407,27 +1407,27 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>BB_AC333_GL</t>
+          <t>ALLUIMINANKRO_R</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>2026-05-06 09:09:45</t>
+          <t>2026-05-06 10:13:22</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>00:56:46</t>
+          <t>00:51:40</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1439,17 +1439,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>AC965</t>
+          <t>ET509</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DIOGOBOUA</t>
+          <t>ATTINGUIE_ZONE_2</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -1459,22 +1459,22 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>AC965_900</t>
+          <t>BB_ET509_GL</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>BTS OUTAGE ERIC</t>
+          <t>Heartbeat Failure</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>2026-05-06 09:26:09</t>
+          <t>2026-05-06 10:16:51</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>00:40:22</t>
+          <t>00:48:11</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -1491,17 +1491,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>ET567</t>
+          <t>ET535</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>BKE_CAMPUS2</t>
+          <t>GONZAGUE_AIR_FRANCE</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>BKE_CAMPUS2</t>
+          <t>GONZAG_AIR_FRANCE</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1521,12 +1521,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>2026-05-06 09:30:23</t>
+          <t>2026-05-06 10:40:13</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>00:36:08</t>
+          <t>00:24:49</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -1543,17 +1543,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ET476</t>
+          <t>ET694</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>KONDOUKRO</t>
+          <t>PBOUET_CITE_GRACE</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1563,22 +1563,22 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>ET476</t>
+          <t>PBOUET_CITE_GRACE</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>CSL Fault</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>2026-05-06 09:54:09</t>
+          <t>2026-05-06 10:40:13</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>00:12:22</t>
+          <t>00:24:49</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -1595,17 +1595,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ET019</t>
+          <t>AC845</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>BLACK_MARKET</t>
+          <t>GNIPI_2</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1615,49 +1615,49 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>BB_ET019_GL</t>
+          <t>AC845</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>BTS OUTAGE HUA</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>2026-05-06 09:54:55</t>
+          <t>2026-05-06 10:41:32</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>00:11:36</t>
+          <t>00:23:30</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>NO DG</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SAN-PEDRO</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>AC858</t>
+          <t>IM023</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DOBA</t>
+          <t>BKE_RTE_KATIOLA</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1667,22 +1667,22 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>AC858</t>
+          <t>BKE_RTE_KATIOLA</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>BTS OUTAGE HUA</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>2026-05-06 10:01:50</t>
+          <t>2026-05-06 10:51:22</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>00:04:41</t>
+          <t>00:13:40</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1692,24 +1692,24 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>NO DG</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MAN</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>IM289</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>KOLIKO</t>
+          <t>PARA</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1719,27 +1719,27 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>KOLIKO</t>
+          <t>ET178</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>BTS OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>2026-05-06 10:04:50</t>
+          <t>2026-05-06 10:55:47</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>00:01:41</t>
+          <t>00:11:45</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -1751,42 +1751,42 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ET452</t>
+          <t>ET425</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>TAKIKRO</t>
+          <t>KOUWEIT_PIERRE_GADIE</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>BB_ET452_W</t>
+          <t>ET425_900</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>NODEB OUTAGE ERIC</t>
+          <t>BTS OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>2026-05-05 00:40:47</t>
+          <t>2026-05-06 10:57:59</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>42:40:01</t>
+          <t>00:07:03</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -1803,47 +1803,47 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>ET063</t>
+          <t>IM289</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>COCODY_MAIRIE</t>
+          <t>KOLIKO</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>BB_ET063_W</t>
+          <t>IM289</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>BTS OUTAGE HUA</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>2026-05-05 15:23:47</t>
+          <t>2026-05-06 11:00:31</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>18:42:44</t>
+          <t>00:04:31</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -1855,42 +1855,42 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>IM011</t>
+          <t>AC044</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>KOBAKRO_ISRAEL</t>
+          <t>OASIS</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>BB_IM011_GW</t>
+          <t>AC044_EXP</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>BTS OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>2026-05-05 15:53:51</t>
+          <t>2026-05-06 11:00:59</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>18:12:40</t>
+          <t>00:04:03</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -1907,42 +1907,42 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>AC350</t>
+          <t>AC704</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>AKOUEDO</t>
+          <t>MAMIE_ADJOUA</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>3G</t>
+          <t>2G</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>BB_AC350_W</t>
+          <t>AC704_900</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>BTS OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>2026-05-05 16:54:09</t>
+          <t>2026-05-06 11:00:59</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>17:12:22</t>
+          <t>00:04:03</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -1959,17 +1959,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>IM036</t>
+          <t>ET063</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>SEGUELA_RTE_BOLO</t>
+          <t>COCODY_MAIRIE</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1979,27 +1979,27 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>SEGUELA_ROUTE_BOLO</t>
+          <t>BB_ET063_W</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>Heartbeat Failure</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>2026-05-05 20:04:10</t>
+          <t>2026-05-05 15:23:47</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>14:02:21</t>
+          <t>19:41:15</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -2011,17 +2011,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>AC943</t>
+          <t>IM011</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>CARR_SEGUELA</t>
+          <t>KOBAKRO_ISRAEL</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -2031,27 +2031,27 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>CARR_SEGUELA</t>
+          <t>BB_IM011_GW</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>Heartbeat Failure</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>2026-05-05 20:04:33</t>
+          <t>2026-05-05 15:53:51</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>14:01:58</t>
+          <t>19:11:11</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -2063,17 +2063,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ABIDJAN 01</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AC414</t>
+          <t>AC350</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>SOLIBRA</t>
+          <t>AKOUEDO</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -2083,7 +2083,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>WAC414</t>
+          <t>BB_AC350_W</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -2093,12 +2093,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>2026-05-05 21:08:33</t>
+          <t>2026-05-05 16:54:09</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>12:57:58</t>
+          <t>18:10:53</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2120,12 +2120,12 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>IM036</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>SEGUELA_RTE_BOLO</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>SEGUELA_ROUTE_BOLO</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -2145,12 +2145,12 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>2026-05-05 22:36:33</t>
+          <t>2026-05-05 20:04:10</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>11:29:58</t>
+          <t>15:00:52</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -2160,24 +2160,24 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>NO DG</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>IM037</t>
+          <t>AC943</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SONGON_KASSAMBLE</t>
+          <t>CARR_SEGUELA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -2187,27 +2187,27 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>BB_IM037_GW</t>
+          <t>CARR_SEGUELA</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>2026-05-06 00:36:02</t>
+          <t>2026-05-05 20:04:33</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>11:15:57</t>
+          <t>15:00:29</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -2219,17 +2219,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>ET803</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ABOBO_AVOCATIER_2 CHATEAUX</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2239,49 +2239,49 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>BB_ET803_W</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>2026-05-06 04:19:38</t>
+          <t>2026-05-05 22:36:33</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>05:46:53</t>
+          <t>12:28:29</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>NO DG</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>AC178</t>
+          <t>IM037</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AGNIKRO</t>
+          <t>SONGON_KASSAMBLE</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -2291,7 +2291,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>BB_AC178_W</t>
+          <t>BB_IM037_GW</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -2301,12 +2301,12 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>2026-05-06 05:17:16</t>
+          <t>2026-05-06 00:36:02</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>04:49:15</t>
+          <t>12:14:28</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -2316,24 +2316,24 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>NO DG</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>IM255</t>
+          <t>ET803</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ATTINGUIE_CANAAN</t>
+          <t>ABOBO_AVOCATIER_2 CHATEAUX</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -2343,7 +2343,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>BB_IM255_GW</t>
+          <t>BB_ET803_W</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -2353,12 +2353,12 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2026-05-06 06:33:03</t>
+          <t>2026-05-06 04:19:38</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>03:33:28</t>
+          <t>06:45:24</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -2375,17 +2375,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ET504</t>
+          <t>IM255</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>ZEPREGUHE</t>
+          <t>ATTINGUIE_CANAAN</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -2395,27 +2395,27 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>ZEBREZIHE</t>
+          <t>BB_IM255_GW</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>Heartbeat Failure</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>2026-05-06 06:38:09</t>
+          <t>2026-05-06 06:33:03</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>03:28:22</t>
+          <t>04:31:59</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -2427,17 +2427,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>AC137</t>
+          <t>ET416</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>DAL_ESCADRON</t>
+          <t>SAGBE_CELESTE</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2447,27 +2447,27 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>DAL_ESCADRON</t>
+          <t>WET416</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>Heartbeat Failure</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>2026-05-06 06:56:41</t>
+          <t>2026-05-06 07:15:15</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>03:09:50</t>
+          <t>04:01:05</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -2479,17 +2479,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ET416</t>
+          <t>AC334</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>SAGBE_CELESTE</t>
+          <t>STIF</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2499,7 +2499,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>WET416</t>
+          <t>WAC334</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
@@ -2509,12 +2509,12 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>2026-05-06 07:15:15</t>
+          <t>2026-05-06 07:59:19</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>03:02:34</t>
+          <t>03:05:43</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -2524,24 +2524,24 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>NO DG</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ET816</t>
+          <t>ET402</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>MASSADOUGOU_EST</t>
+          <t>ADJAME_UTB</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>BB_ET816_W</t>
+          <t>BB_ET402_W</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
@@ -2561,12 +2561,12 @@
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2026-05-06 07:30:41</t>
+          <t>2026-05-06 08:00:41</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>02:35:50</t>
+          <t>03:04:21</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -2588,12 +2588,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>AC334</t>
+          <t>AC333</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>STIF</t>
+          <t>DJEDA</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2603,7 +2603,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>WAC334</t>
+          <t>BB_AC333_W</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2613,12 +2613,12 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-05-06 07:59:19</t>
+          <t>2026-05-06 09:11:03</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>02:07:12</t>
+          <t>01:53:59</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -2628,24 +2628,24 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>NO DG</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>ET402</t>
+          <t>AC965</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ADJAME_UTB</t>
+          <t>DIOGOBOUA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -2655,7 +2655,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>BB_ET402_W</t>
+          <t>BB_AC965_W</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2665,12 +2665,12 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>2026-05-06 08:00:41</t>
+          <t>2026-05-06 09:29:35</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>02:05:50</t>
+          <t>01:49:01</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -2680,24 +2680,24 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>NO DG</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ET350</t>
+          <t>ET567</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>BOUAFLE_HERE</t>
+          <t>BKE_CAMPUS2</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -2707,7 +2707,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>BOUAFLE_HERE</t>
+          <t>BKE_CAMPUS2</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
@@ -2717,12 +2717,12 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>2026-05-06 08:49:23</t>
+          <t>2026-05-06 09:30:23</t>
         </is>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>01:17:08</t>
+          <t>01:34:39</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -2744,12 +2744,12 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>AC333</t>
+          <t>AC726</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>DJEDA</t>
+          <t>ANGRE_PRGRME6</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -2759,22 +2759,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>BB_AC333_W</t>
+          <t>BB_AC726_W</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NODEB OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>2026-05-06 09:11:03</t>
+          <t>2026-05-06 09:33:39</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>00:55:28</t>
+          <t>01:31:26</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
@@ -2791,17 +2791,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>AC965</t>
+          <t>ET019</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>DIOGOBOUA</t>
+          <t>BLACK_MARKET</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -2811,7 +2811,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>BB_AC965_W</t>
+          <t>WET019</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2821,12 +2821,12 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>2026-05-06 09:29:35</t>
+          <t>2026-05-06 09:54:03</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>00:50:30</t>
+          <t>01:10:59</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -2836,24 +2836,24 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>NO DG</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ET567</t>
+          <t>ET517</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>BKE_CAMPUS2</t>
+          <t>ADJAME RENAULT</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -2863,27 +2863,27 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>BKE_CAMPUS2</t>
+          <t>BB_ET517_W</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>NODEB OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>2026-05-06 09:30:23</t>
+          <t>2026-05-06 10:00:38</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>00:36:08</t>
+          <t>01:04:24</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
@@ -2895,17 +2895,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>AC726</t>
+          <t>ET641</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>ANGRE_PRGRME6</t>
+          <t>DIANGOBO</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2915,22 +2915,22 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>BB_AC726_W</t>
+          <t>BB_ET641_W</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>NODEB OUTAGE ERIC</t>
+          <t>Heartbeat Failure</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>2026-05-06 09:33:39</t>
+          <t>2026-05-06 10:04:20</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>00:32:55</t>
+          <t>01:00:42</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
@@ -2947,17 +2947,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>MAN</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ET019</t>
+          <t>IM289</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BLACK_MARKET</t>
+          <t>KOLIKO</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -2967,27 +2967,27 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>WET019</t>
+          <t>KOLIKO</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>2026-05-06 09:54:03</t>
+          <t>2026-05-06 10:04:50</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>00:12:28</t>
+          <t>01:00:12</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -2999,17 +2999,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>YAMOUSSOUKRO</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ET381</t>
+          <t>IM398</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CAFETOU</t>
+          <t>RURAL_ALLUIMINANKRO</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -3019,27 +3019,27 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>WET381</t>
+          <t>ALLUIMINANKRO_R</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>NODEB OUTAGE ERIC</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>2026-05-06 10:00:00</t>
+          <t>2026-05-06 10:13:22</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>00:06:31</t>
+          <t>00:51:40</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -3051,27 +3051,27 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ET063</t>
+          <t>ET509</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>COCODY_MAIRIE</t>
+          <t>ATTINGUIE_ZONE_2</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>BB_ET063_GL</t>
+          <t>BB_ET509_W</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
@@ -3081,12 +3081,12 @@
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>2026-05-05 15:24:43</t>
+          <t>2026-05-06 10:17:29</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>18:41:48</t>
+          <t>00:47:33</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -3096,54 +3096,54 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>NO DG</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>IM011</t>
+          <t>ET535</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>KOBAKRO_ISRAEL</t>
+          <t>GONZAGUE_AIR_FRANCE</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>BB_IM011_L</t>
+          <t>GONZAG_AIR_FRANCE</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>2026-05-05 15:53:50</t>
+          <t>2026-05-06 10:40:13</t>
         </is>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>18:12:41</t>
+          <t>00:24:49</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
@@ -3155,47 +3155,47 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 01</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>AC350</t>
+          <t>ET694</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>AKOUEDO</t>
+          <t>PBOUET_CITE_GRACE</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>BB_AC350_GL</t>
+          <t>PBOUET_CITE_GRACE</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>2026-05-05 16:54:05</t>
+          <t>2026-05-06 10:40:13</t>
         </is>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>17:12:26</t>
+          <t>00:24:49</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
@@ -3207,42 +3207,42 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>SAN-PEDRO</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>IM036</t>
+          <t>AC845</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>SEGUELA_RTE_BOLO</t>
+          <t>GNIPI_2</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>SEGUELA_ROUTE_BOLO</t>
+          <t>WAC845</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>NODEB OUTAGE HUA</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>2026-05-05 20:04:10</t>
+          <t>2026-05-06 10:41:38</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>14:02:21</t>
+          <t>00:23:38</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -3252,34 +3252,34 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>NO DG</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>BOUAKE</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>AC943</t>
+          <t>IM023</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>CARR_SEGUELA</t>
+          <t>BKE_RTE_KATIOLA</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>CARR_SEGUELA</t>
+          <t>BKE_RTE_KATIOLA</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -3289,12 +3289,12 @@
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>2026-05-05 20:04:33</t>
+          <t>2026-05-06 10:51:22</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>14:01:58</t>
+          <t>00:13:40</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -3311,47 +3311,47 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>AC827</t>
+          <t>ET233</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>SAPH_SAIBE</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>DANIA</t>
+          <t>BB_ET233_W</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>NODEB OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>2026-05-05 22:36:33</t>
+          <t>2026-05-06 10:59:32</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>11:29:58</t>
+          <t>00:05:30</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
@@ -3363,42 +3363,42 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>ET803</t>
+          <t>AC516</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ABOBO_AVOCATIER_2 CHATEAUX</t>
+          <t>BETTIE</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>BB_ET803_GL</t>
+          <t>WAC516</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NODEB OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>2026-05-06 04:19:07</t>
+          <t>2026-05-06 10:59:32</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>05:47:24</t>
+          <t>00:05:30</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -3408,54 +3408,54 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>NO DG</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>GAGNOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>ET702</t>
+          <t>AC704</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ROA</t>
+          <t>MAMIE_ADJOUA</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>LET702</t>
+          <t>BB_AC704_W</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>ENODEB OUTAGE HUA</t>
+          <t>NODEB OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>2026-05-06 04:19:34</t>
+          <t>2026-05-06 11:00:17</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>05:46:57</t>
+          <t>00:04:45</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
@@ -3467,42 +3467,42 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>AC178</t>
+          <t>ET389</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>AGNIKRO</t>
+          <t>MAROC_ANTENNE</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>BB_AC178_GL</t>
+          <t>BB_ET389_W</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NODEB OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>2026-05-06 05:19:21</t>
+          <t>2026-05-06 11:00:17</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>04:47:10</t>
+          <t>00:04:45</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -3512,49 +3512,49 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>NO DG</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABENGOUROU</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>IM255</t>
+          <t>ET232</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ATTINGUIE_CANAAN</t>
+          <t>ABRADINOU</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>BB_IM255_L</t>
+          <t>BB_ET232_W</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NODEB OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>2026-05-06 06:33:01</t>
+          <t>2026-05-06 11:02:14</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>03:33:30</t>
+          <t>00:02:48</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -3571,47 +3571,47 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>ET504</t>
+          <t>AC044</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>ZEPREGUHE</t>
+          <t>OASIS</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>4G</t>
+          <t>3G</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>ZEBREZIHE</t>
+          <t>WAC044</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>NODEB OUTAGE ERIC</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>2026-05-06 06:38:09</t>
+          <t>2026-05-06 11:02:57</t>
         </is>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>03:28:22</t>
+          <t>00:02:05</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J62" t="inlineStr">
@@ -3623,17 +3623,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>DALOA</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>AC137</t>
+          <t>ET063</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>DAL_ESCADRON</t>
+          <t>COCODY_MAIRIE</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -3643,27 +3643,27 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>DAL_ESCADRON</t>
+          <t>BB_ET063_GL</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>Heartbeat Failure</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>2026-05-06 06:56:41</t>
+          <t>2026-05-05 15:24:43</t>
         </is>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>03:09:50</t>
+          <t>19:40:19</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J63" t="inlineStr">
@@ -3675,17 +3675,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>ET584</t>
+          <t>IM011</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>PRUNELLE_JACQUEVIL</t>
+          <t>KOBAKRO_ISRAEL</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -3695,7 +3695,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>BB_ET584_GL</t>
+          <t>BB_IM011_L</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3705,12 +3705,12 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>2026-05-06 07:10:24</t>
+          <t>2026-05-05 15:53:50</t>
         </is>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>03:41:50</t>
+          <t>19:11:12</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -3727,17 +3727,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>ABIDJAN 04</t>
+          <t>ABIDJAN 03</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>ET416</t>
+          <t>AC350</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>SAGBE_CELESTE</t>
+          <t>AKOUEDO</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -3747,7 +3747,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>BB_ET416_GL</t>
+          <t>BB_AC350_GL</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -3757,12 +3757,12 @@
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>2026-05-06 07:18:08</t>
+          <t>2026-05-05 16:54:05</t>
         </is>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>02:48:23</t>
+          <t>18:10:57</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -3779,17 +3779,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ABENGOUROU</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>ET816</t>
+          <t>IM036</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>MASSADOUGOU_EST</t>
+          <t>SEGUELA_RTE_BOLO</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -3799,27 +3799,27 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>BB_ET816_GL</t>
+          <t>SEGUELA_ROUTE_BOLO</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>2026-05-06 07:29:58</t>
+          <t>2026-05-05 20:04:10</t>
         </is>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>02:36:33</t>
+          <t>15:00:52</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="J66" t="inlineStr">
@@ -3831,17 +3831,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>AC334</t>
+          <t>AC943</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>STIF</t>
+          <t>CARR_SEGUELA</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -3851,49 +3851,49 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>BB_AC334_GL</t>
+          <t>CARR_SEGUELA</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>2026-05-06 08:00:27</t>
+          <t>2026-05-05 20:04:33</t>
         </is>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>02:06:04</t>
+          <t>15:00:29</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>DG</t>
+          <t>NO DG</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>DALOA</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>ET402</t>
+          <t>AC827</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>ADJAME_UTB</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -3903,49 +3903,49 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>BB_ET402_GL</t>
+          <t>DANIA</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Heartbeat Failure</t>
+          <t>NE Is Disconnected</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>2026-05-06 08:02:43</t>
+          <t>2026-05-05 22:36:33</t>
         </is>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>02:03:48</t>
+          <t>12:28:29</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>ERICSSON</t>
+          <t>HUAWEI</t>
         </is>
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>NO DG</t>
+          <t>DG</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ABIDJAN 02</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>ET293</t>
+          <t>ET803</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>NDJEM</t>
+          <t>ABOBO_AVOCATIER_2 CHATEAUX</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -3955,22 +3955,22 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>BB_ET293_GL</t>
+          <t>BB_ET803_GL</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>ENODEB OUTAGE ERIC</t>
+          <t>Heartbeat Failure</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>2026-05-06 08:37:47</t>
+          <t>2026-05-06 04:19:07</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>01:31:09</t>
+          <t>06:45:55</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -3987,17 +3987,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>YAMOUSSOUKRO</t>
+          <t>GAGNOA</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>ET350</t>
+          <t>ET702</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>BOUAFLE_HERE</t>
+          <t>ROA</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -4007,22 +4007,22 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>BOUAFLE_HERE</t>
+          <t>LET702</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>ENODEB OUTAGE HUA</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>2026-05-06 08:49:23</t>
+          <t>2026-05-06 04:19:34</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>01:17:08</t>
+          <t>06:45:28</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -4039,17 +4039,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>AC333</t>
+          <t>IM255</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>DJEDA</t>
+          <t>ATTINGUIE_CANAAN</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -4059,7 +4059,7 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>BB_AC333_GL</t>
+          <t>BB_IM255_L</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -4069,12 +4069,12 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>2026-05-06 09:09:45</t>
+          <t>2026-05-06 06:33:01</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>00:56:46</t>
+          <t>04:32:01</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -4091,17 +4091,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BOUAKE</t>
+          <t>ABIDJAN 02</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>ET567</t>
+          <t>ET584</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>BKE_CAMPUS2</t>
+          <t>PRUNELLE_JACQUEVIL</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -4111,27 +4111,27 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>BKE_CAMPUS2</t>
+          <t>BB_ET584_GL</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>NE Is Disconnected</t>
+          <t>Heartbeat Failure</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>2026-05-06 09:30:23</t>
+          <t>2026-05-06 07:10:24</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>00:36:08</t>
+          <t>04:40:21</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
         <is>
-          <t>HUAWEI</t>
+          <t>ERICSSON</t>
         </is>
       </c>
       <c r="J72" t="inlineStr">
@@ -4143,17 +4143,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ABIDJAN 03</t>
+          <t>ABIDJAN 04</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>ET019</t>
+          <t>ET416</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>BLACK_MARKET</t>
+          <t>SAGBE_CELESTE</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -4163,7 +4163,7 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>BB_ET019_GL</t>
+          <t>BB_ET416_GL</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
@@ -4173,12 +4173,12 @@
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>2026-05-06 09:54:55</t>
+          <t>2026-05-06 07:18:08</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>00:11:36</t>
+          <t>03:46:54</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -4195,52 +4195,676 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
+          <t>ABIDJAN 03</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>AC334</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>STIF</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>BB_AC334_GL</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Heartbeat Failure</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2026-05-06 08:00:27</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>03:04:35</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>DG</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>ABIDJAN 03</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ET402</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>ADJAME_UTB</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>BB_ET402_GL</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Heartbeat Failure</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2026-05-06 08:02:43</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>03:02:19</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>NO DG</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ET293</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>NDJEM</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>BB_ET293_GL</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>ENODEB OUTAGE ERIC</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2026-05-06 08:37:47</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>02:29:40</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>NO DG</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>ABIDJAN 03</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>AC333</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>DJEDA</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>BB_AC333_GL</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Heartbeat Failure</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2026-05-06 09:09:45</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>01:55:17</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>NO DG</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>BOUAKE</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>ET567</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>BKE_CAMPUS2</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>BKE_CAMPUS2</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>NE Is Disconnected</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2026-05-06 09:30:23</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>01:34:39</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>HUAWEI</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>NO DG</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>ABIDJAN 03</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ET019</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>BLACK_MARKET</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>BB_ET019_GL</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Heartbeat Failure</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2026-05-06 09:54:55</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>01:10:07</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>NO DG</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>ABIDJAN 04</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>ET641</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>DIANGOBO</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>BB_ET641_GL</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Heartbeat Failure</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2026-05-06 10:04:22</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>01:00:40</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>NO DG</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>MAN</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>IM289</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>KOLIKO</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>KOLIKO</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>NE Is Disconnected</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2026-05-06 10:04:50</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>01:00:12</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>HUAWEI</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>NO DG</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
           <t>YAMOUSSOUKRO</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>AC122</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>YAM_DAUPHIN</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>IM398</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>RURAL_ALLUIMINANKRO</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
         <is>
           <t>4G</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>LAC122</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>ENODEB OUTAGE HUA</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>2026-05-06 10:01:01</t>
-        </is>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>00:05:30</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>ALLUIMINANKRO_R</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>NE Is Disconnected</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2026-05-06 10:13:22</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>00:51:40</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
         <is>
           <t>HUAWEI</t>
         </is>
       </c>
-      <c r="J74" t="inlineStr">
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>NO DG</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>ABIDJAN 02</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>ET509</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>ATTINGUIE_ZONE_2</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>BB_ET509_GL</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Heartbeat Failure</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2026-05-06 10:16:51</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>00:48:11</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>ERICSSON</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
         <is>
           <t>DG</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>ABIDJAN 01</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>ET535</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>GONZAGUE_AIR_FRANCE</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>GONZAG_AIR_FRANCE</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>NE Is Disconnected</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2026-05-06 10:40:13</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>00:24:49</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>HUAWEI</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>NO DG</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>ABIDJAN 01</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>ET694</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>PBOUET_CITE_GRACE</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>PBOUET_CITE_GRACE</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>NE Is Disconnected</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2026-05-06 10:40:13</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>00:24:49</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>HUAWEI</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>NO DG</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>BOUAKE</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>IM023</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>BKE_RTE_KATIOLA</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>4G</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>BKE_RTE_KATIOLA</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>NE Is Disconnected</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2026-05-06 10:51:22</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>00:13:40</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>HUAWEI</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>NO DG</t>
         </is>
       </c>
     </row>

</xml_diff>